<commit_message>
feat(km19): dong bo ho so thuc te 11 sheet tan suat, 6 bang boc tach CAD nhung so do PNG va tai lieu README
</commit_message>
<xml_diff>
--- a/examples/HO_SO_CAU_KM19_529/03_KINH_TE_QS_DU_TOAN_THANH_TOAN/03_QS_Dien_Giai_Chi_Tiet_Takeoff.xlsx
+++ b/examples/HO_SO_CAU_KM19_529/03_KINH_TE_QS_DU_TOAN_THANH_TOAN/03_QS_Dien_Giai_Chi_Tiet_Takeoff.xlsx
@@ -419,6 +419,166 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>13</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="12858750" cy="7505700"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>13</col>
+      <colOff>0</colOff>
+      <row>35</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="12858750" cy="7419975"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>13</col>
+      <colOff>0</colOff>
+      <row>67</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="12858750" cy="7915275"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>13</col>
+      <colOff>0</colOff>
+      <row>99</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="12858750" cy="8572500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>11</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="12858750" cy="7505700"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>11</col>
+      <colOff>0</colOff>
+      <row>35</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="12858750" cy="7505700"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -708,7 +868,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L101"/>
+  <dimension ref="A2:L101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -725,7 +885,6 @@
     <col width="18" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -4156,6 +4315,7 @@
     <mergeCell ref="A6:L6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4165,7 +4325,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A2:J21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4180,7 +4340,6 @@
     <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -4826,7 +4985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q408"/>
+  <dimension ref="A2:Q408"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4848,7 +5007,6 @@
     <col width="25" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -32776,7 +32934,6 @@
         </is>
       </c>
     </row>
-    <row r="401"/>
     <row r="402">
       <c r="B402" s="30" t="inlineStr">
         <is>
@@ -33367,5 +33524,6 @@
     <mergeCell ref="A2:J2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>